<commit_message>
CoS-014, CoS-017, CoS-018, CoS-019, DC-026
</commit_message>
<xml_diff>
--- a/docs/kostenuebersicht-finance.xlsx
+++ b/docs/kostenuebersicht-finance.xlsx
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="198">
   <si>
     <t xml:space="preserve">Sofortangebot — Laufende Geschäftskosten</t>
   </si>
@@ -309,10 +309,7 @@
     <t xml:space="preserve">USt. direkt ausgewiesen (EU OSS VAT EU372041333), kein Reverse Charge</t>
   </si>
   <si>
-    <t xml:space="preserve">auffällig — falscher Account?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 Beleg (Journal 2026-004) vom 14.06.2026 über $15,00 + USt = $17,85. Rechnungsempfänger 'Hugo' / runningwithhugo@outlook.de — andere Identität als bei den übrigen Diensten.</t>
+    <t xml:space="preserve">1 Beleg (Journal 2026-004) vom 14.06.2026 über $15,00 + USt = $17,85. Rechnungsempfänger 'Hugo' / runningwithhugo@outlook.de — ist Sandys eigener Account, Name/E-Mail-Alias lässt sich bei OpenAI nachträglich nicht mehr ändern (geklärt 19.08.2026).</t>
   </si>
   <si>
     <t xml:space="preserve">Resend</t>
@@ -558,7 +555,7 @@
     <t xml:space="preserve">Invoice-YL9K6L19-0001.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">Rechnungsempfänger 'Hugo' / andere E-Mail als bei allen übrigen Diensten — bitte prüfen, ob das der richtige Account für Sofortangebot ist.</t>
+    <t xml:space="preserve">Geklärt (19.08.2026): Konto gehört Sandy, 'Hugo' ist ein historischer Nutzername/E-Mail-Alias bei OpenAI, der sich im Nachhinein nicht mehr auf 'Sandra Holm' ändern lässt. Kein falscher Account — nur zur Info für den Steuerberater vermerkt, falls Name/E-Mail auf dem Beleg auffallen.</t>
   </si>
   <si>
     <t xml:space="preserve">2026-005</t>
@@ -751,9 +748,6 @@
   </si>
   <si>
     <t xml:space="preserve">• Claude-Pro-Apple-Abo: Belege für Juni und Juli fehlen (nur Mai und August vorhanden) — bitte in der Apple-Kaufhistorie nachsehen und ergänzen, damit der Monatsverlauf vollständig ist.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• OpenAI-Beleg ist auf 'Hugo' / runningwithhugo@outlook.de ausgestellt, nicht auf Sandra Holm / einfachanfrage@outlook.com wie die anderen Dienste. Richtiger Account?</t>
   </si>
   <si>
     <t xml:space="preserve">• Zwei unterschiedliche Adressen für Sandra Holm (Wielandstraße 11 vs. Krampasplatz 4b) — vermutlich alt/neu, bitte kurz bestätigen.</t>
@@ -1599,7 +1593,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>41</v>
       </c>
@@ -1609,7 +1603,7 @@
       <c r="C9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="7" t="n">
         <v>17.85</v>
       </c>
       <c r="E9" s="4" t="s">
@@ -1621,22 +1615,22 @@
       <c r="G9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="H9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="D10" s="9"/>
       <c r="E10" s="4" t="s">
@@ -1649,48 +1643,48 @@
         <v>29</v>
       </c>
       <c r="H10" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>52</v>
-      </c>
       <c r="C11" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D11" s="9"/>
       <c r="E11" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>54</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>29</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>57</v>
-      </c>
       <c r="C12" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D12" s="9"/>
       <c r="E12" s="4" t="s">
@@ -1703,25 +1697,25 @@
         <v>29</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="C13" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>29</v>
@@ -1730,37 +1724,37 @@
         <v>29</v>
       </c>
       <c r="H13" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="I13" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="4" t="s">
-        <v>65</v>
-      </c>
       <c r="C14" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>66</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>29</v>
       </c>
       <c r="H14" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="I14" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,7 +1781,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -1803,7 +1797,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -1819,7 +1813,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1874,7 +1868,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1897,7 +1891,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1920,84 +1914,84 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>80</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="O4" s="3" t="s">
+      <c r="P4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="P4" s="3" t="s">
+      <c r="Q4" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="Q4" s="3" t="s">
+      <c r="R4" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="16" t="n">
         <v>46146</v>
       </c>
       <c r="C5" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>95</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>33</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>35</v>
@@ -2015,46 +2009,46 @@
         <v>22</v>
       </c>
       <c r="N5" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O5" s="19" t="n">
         <f aca="false">M5</f>
         <v>22</v>
       </c>
       <c r="P5" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="R5" s="20" t="s">
         <v>99</v>
-      </c>
-      <c r="R5" s="20" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B6" s="16" t="n">
         <v>46164</v>
       </c>
       <c r="C6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="E6" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>13</v>
@@ -2072,41 +2066,41 @@
         <v>23.8</v>
       </c>
       <c r="N6" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O6" s="21"/>
       <c r="P6" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q6" s="4" t="s">
         <v>108</v>
-      </c>
-      <c r="Q6" s="4" t="s">
-        <v>109</v>
       </c>
       <c r="R6" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B7" s="16" t="n">
         <v>46165</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>13</v>
@@ -2115,7 +2109,7 @@
         <v>25</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>0</v>
@@ -2124,43 +2118,43 @@
         <v>25</v>
       </c>
       <c r="N7" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O7" s="21"/>
       <c r="P7" s="4" t="s">
         <v>29</v>
       </c>
       <c r="Q7" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="R7" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="R7" s="20" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
         <v>119</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>120</v>
       </c>
       <c r="B8" s="16" t="n">
         <v>46187</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>123</v>
-      </c>
       <c r="F8" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>41</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>13</v>
@@ -2178,43 +2172,43 @@
         <v>17.85</v>
       </c>
       <c r="N8" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="O8" s="21"/>
       <c r="P8" s="4" t="s">
         <v>29</v>
       </c>
       <c r="Q8" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="R8" s="20" t="s">
         <v>126</v>
-      </c>
-      <c r="R8" s="20" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B9" s="16" t="n">
         <v>46195</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>130</v>
-      </c>
       <c r="E9" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>13</v>
@@ -2232,43 +2226,43 @@
         <v>23.8</v>
       </c>
       <c r="N9" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O9" s="21"/>
       <c r="P9" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q9" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="R9" s="20" t="s">
         <v>131</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B10" s="16" t="n">
         <v>46196</v>
       </c>
       <c r="C10" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>135</v>
-      </c>
       <c r="E10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>13</v>
@@ -2277,7 +2271,7 @@
         <v>49.97</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>0</v>
@@ -2286,43 +2280,43 @@
         <v>49.97</v>
       </c>
       <c r="N10" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O10" s="21"/>
       <c r="P10" s="4" t="s">
         <v>29</v>
       </c>
       <c r="Q10" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="R10" s="20" t="s">
         <v>136</v>
-      </c>
-      <c r="R10" s="20" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B11" s="16" t="n">
         <v>46225</v>
       </c>
       <c r="C11" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>140</v>
-      </c>
       <c r="E11" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>104</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>105</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>13</v>
@@ -2340,41 +2334,41 @@
         <v>23.8</v>
       </c>
       <c r="N11" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O11" s="21"/>
       <c r="P11" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q11" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="R11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B12" s="16" t="n">
         <v>46226</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>144</v>
-      </c>
       <c r="E12" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>114</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>13</v>
@@ -2383,7 +2377,7 @@
         <v>54.3</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>0</v>
@@ -2392,43 +2386,43 @@
         <v>54.3</v>
       </c>
       <c r="N12" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="O12" s="21"/>
       <c r="P12" s="4" t="s">
         <v>29</v>
       </c>
       <c r="Q12" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="R12" s="20" t="s">
         <v>145</v>
-      </c>
-      <c r="R12" s="20" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B13" s="16" t="n">
         <v>46237</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>149</v>
-      </c>
       <c r="E13" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>94</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>95</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>33</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>35</v>
@@ -2446,46 +2440,46 @@
         <v>22</v>
       </c>
       <c r="N13" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="O13" s="19" t="n">
         <f aca="false">M13</f>
         <v>22</v>
       </c>
       <c r="P13" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="Q13" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="R13" s="20" t="s">
         <v>150</v>
-      </c>
-      <c r="R13" s="20" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B14" s="16" t="n">
         <v>46251</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>154</v>
-      </c>
       <c r="F14" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>13</v>
@@ -2503,17 +2497,17 @@
         <v>53.55</v>
       </c>
       <c r="N14" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="O14" s="21"/>
       <c r="P14" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q14" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="R14" s="20" t="s">
         <v>157</v>
-      </c>
-      <c r="R14" s="20" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2947,7 +2941,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2961,7 +2955,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2978,31 +2972,31 @@
         <v>2</v>
       </c>
       <c r="B4" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="C4" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="D4" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="E4" s="24" t="s">
         <v>163</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="F4" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="F4" s="24" t="s">
+      <c r="G4" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="G4" s="24" t="s">
+      <c r="H4" s="24" t="s">
         <v>166</v>
       </c>
-      <c r="H4" s="24" t="s">
+      <c r="I4" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="I4" s="24" t="s">
+      <c r="J4" s="25" t="s">
         <v>168</v>
-      </c>
-      <c r="J4" s="25" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3212,7 +3206,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="31"/>
       <c r="C10" s="31"/>
@@ -3229,7 +3223,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="31"/>
       <c r="C11" s="31"/>
@@ -3246,7 +3240,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="31"/>
@@ -3263,7 +3257,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="31"/>
@@ -3280,7 +3274,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="31"/>
       <c r="C14" s="31"/>
@@ -3297,7 +3291,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B16" s="14" t="n">
         <f aca="false">IF(B5="",0,B5)+IF(B6="",0,B6)+IF(B7="",0,B7)+IF(B9="",0,B9)</f>
@@ -3335,7 +3329,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">IF(B8="",0,B8)</f>
@@ -3391,7 +3385,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -3399,142 +3393,137 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="34" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="35" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="35" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="36" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="36" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="36" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="36" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="36" t="s">
         <v>194</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="36" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="36" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="36" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="36" t="s">
+    <row r="33" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="42" t="s">
         <v>197</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="36" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="42" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Pruefmeister: vier Haken zurueckgezogen (PM-002/006/010/018), sechs VOB-Fragen beantwortet, VOB-014 Paketaufrundung
</commit_message>
<xml_diff>
--- a/docs/kostenuebersicht-finance.xlsx
+++ b/docs/kostenuebersicht-finance.xlsx
@@ -62,7 +62,7 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
-    <comment ref="A15" authorId="0">
+    <comment ref="A22" authorId="0">
       <text>
         <r>
           <rPr>
@@ -70,11 +70,35 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Ab hier: freie Zeilen für neue Belege. Bitte fortlaufende Beleg-Nr. vergeben (z. B. 2026-011) und nie bestehende Zeilen überschreiben/löschen.</t>
+          <t xml:space="preserve">Ab hier: freie Zeilen für neue Belege. Bitte fortlaufende Beleg-Nr. vergeben (z. B. 2026-018) und nie bestehende Zeilen überschreiben/löschen.</t>
         </r>
       </text>
     </comment>
-    <comment ref="O6" authorId="0">
+    <comment ref="N15" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Rechnung bündelt mehrere Domains/Positionen unter einer Vertragsnummer — dieser Betrag ist nur der Sofortangebot-Anteil (Brutto), nicht die volle Rechnungssumme. Details in der Notiz-Spalte. Monatsverlauf summiert nach dieser Spalte, nicht nach Brutto-Betrag.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N16" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Rechnung bündelt mehrere Domains/Positionen unter einer Vertragsnummer — dieser Betrag ist nur der Sofortangebot-Anteil (Brutto), nicht die volle Rechnungssumme. Details in der Notiz-Spalte. Monatsverlauf summiert nach dieser Spalte, nicht nach Brutto-Betrag.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P6" authorId="0">
       <text>
         <r>
           <rPr>
@@ -86,7 +110,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O7" authorId="0">
+    <comment ref="P7" authorId="0">
       <text>
         <r>
           <rPr>
@@ -98,7 +122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O8" authorId="0">
+    <comment ref="P8" authorId="0">
       <text>
         <r>
           <rPr>
@@ -110,7 +134,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O9" authorId="0">
+    <comment ref="P9" authorId="0">
       <text>
         <r>
           <rPr>
@@ -122,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O10" authorId="0">
+    <comment ref="P10" authorId="0">
       <text>
         <r>
           <rPr>
@@ -134,7 +158,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O11" authorId="0">
+    <comment ref="P11" authorId="0">
       <text>
         <r>
           <rPr>
@@ -146,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O12" authorId="0">
+    <comment ref="P12" authorId="0">
       <text>
         <r>
           <rPr>
@@ -158,7 +182,31 @@
         </r>
       </text>
     </comment>
-    <comment ref="O14" authorId="0">
+    <comment ref="P14" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Noch nicht umgerechnet — Umrechnungskurs bewusst nicht erfunden. Bitte mit Steuerberater klären, welcher Stichtags-/Monatskurs für die Buchführung verwendet werden soll (z. B. EZB-Referenzkurs am Rechnungsdatum oder monatlicher BMF-Umrechnungskurs).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P19" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Noch nicht umgerechnet — Umrechnungskurs bewusst nicht erfunden. Bitte mit Steuerberater klären, welcher Stichtags-/Monatskurs für die Buchführung verwendet werden soll (z. B. EZB-Referenzkurs am Rechnungsdatum oder monatlicher BMF-Umrechnungskurs).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P20" authorId="0">
       <text>
         <r>
           <rPr>
@@ -175,12 +223,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="245">
   <si>
     <t xml:space="preserve">Sofortangebot — Laufende Geschäftskosten</t>
   </si>
   <si>
-    <t xml:space="preserve">Stand: 2026-08-19 · Head of Finance · Bestandsaufnahme CoS-F-001 · Beleg-Details je Rechnung stehen im Blatt 'Rechnungsjournal' · orange = auffällig, bitte klären · grau = noch kein Beleg</t>
+    <t xml:space="preserve">Stand: 2026-09-02 · Head of Finance · Bestandsaufnahme CoS-F-001 · Beleg-Details je Rechnung stehen im Blatt 'Rechnungsjournal' · orange = auffällig, bitte klären · grau = noch kein Beleg</t>
   </si>
   <si>
     <t xml:space="preserve">Dienst</t>
@@ -231,7 +279,7 @@
     <t xml:space="preserve">auffällig — Betrag bestätigt, Trend + Projektanzahl bitte klären</t>
   </si>
   <si>
-    <t xml:space="preserve">3 Belege (Journal 2026-003/006/008): 23.05. $25,00 / 23.06. $49,97 / 23.07. $54,30 — steigender Trend. Rechnungen listen 5 Projekt-Referenzen, dokumentiert sind nur 2. Bitte klären, ob alle nötig sind.</t>
+    <t xml:space="preserve">4 Belege (Journal 2026-003/006/008/016): 23.05. $25,00 / 23.06. $49,97 / 23.07. $54,30 / 23.08. $53,83 — nach dem Anstieg jetzt erstmals leicht rückläufig. Rechnungen zeigten bis Juli 5 Projekt-Referenzen, dokumentiert sind nur 2; im August-Beleg taucht eine davon erstmals nicht mehr auf (jetzt 4). Bitte weiter beobachten/klären, ob alle nötig sind.</t>
   </si>
   <si>
     <t xml:space="preserve">Vercel</t>
@@ -252,7 +300,7 @@
     <t xml:space="preserve">bestätigt</t>
   </si>
   <si>
-    <t xml:space="preserve">3 Belege (Journal 2026-002/005/007): 22.05., 22.06., 22.07. — durchgängig $23,80, stabil.</t>
+    <t xml:space="preserve">4 Belege (Journal 2026-002/005/007/015): 22.05., 22.06., 22.07., 22.08. — durchgängig $23,80, stabil. Zahlungsart jetzt bestätigt: Kreditkarte Visa •••3991.</t>
   </si>
   <si>
     <t xml:space="preserve">Anthropic — direkt</t>
@@ -333,13 +381,16 @@
     <t xml:space="preserve">Domain</t>
   </si>
   <si>
-    <t xml:space="preserve">vermutlich jährlich</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Registrar/Ablaufdatum unbekannt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Von Sandy als laufende Kostenposition genannt, noch keine Rechnung im Belege-Ordner.</t>
+    <t xml:space="preserve">'IONOS Mail Basic 5' (Postfach) laufend 2,50 €/Monat. Domain .app + 'Domain Guard' (Privatsphärenschutz) jährlich, zusammen 13,00 € brutto — nächste Fälligkeit ~06/2027.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertragsnummer 111811442 bei IONOS SE — Achtung: bündelt auf denselben Rechnungen auch mehrere fremde Domains, siehe Journal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. direkt von IONOS ausgewiesen (USt-IdNr. DE815563912), kein Reverse Charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 Belege (Journal 2026-011 bis 2026-015/017 — Rechnungsnummern siehe dort) unter einer gebündelten IONOS-Rechnung. Domain sofortangebot.app wurde 08.06.2026 registriert. Sandy hat am 02.09.2026 bestätigt, dass 'Domain Guard' und 'IONOS Mail Basic 5' ebenfalls zu sofortangebot.app gehören. Fremde Domains ('einfach-anfrage.com', 'einfachanfrage-hochzeitsfotografie.de' u. a.) laufen über denselben IONOS-Vertrag, aber NICHT mitgezählt.</t>
   </si>
   <si>
     <t xml:space="preserve">Sentry</t>
@@ -432,6 +483,9 @@
     <t xml:space="preserve">Brutto-Betrag</t>
   </si>
   <si>
+    <t xml:space="preserve">Sofortangebot-Anteil (Brutto)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Steuerliche Einordnung</t>
   </si>
   <si>
@@ -498,159 +552,291 @@
     <t xml:space="preserve">USt. (19%) direkt von Vercel ausgewiesen (EU VAT EU056329113), kein Reverse Charge.</t>
   </si>
   <si>
+    <t xml:space="preserve">Kreditkarte Visa •••3991</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-TT0BDQ8S-0001.pdf / Receipt-2392-5328.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zahlungsart nachträglich ergänzt (Update 2026-09-02) anhand Zahlungsbeleg Receipt-2392-5328.pdf.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVGOOM-00003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.05.–22.06.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supabase Pte. Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Singapur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandra Holm, Wielandstraße 11, Berlin (einfachanfrage@outlook.com)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse Charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse Charge — Supabase weist keine USt aus. Sandy startet als Kleinunternehmerin nach §19 UStG (bestätigt 19.08.2026), Gewerbe aber noch nicht angemeldet. Nach Kleinunternehmerregelung i. d. R. keine Vorsteuer ziehbar, aber die USt-Pflicht auf reverse-charge-Leistungen aus dem Ausland (§13b UStG) kann trotzdem bestehen bleiben — das ist keine verbindliche Auskunft von mir, bitte mit Steuerberater final klären, sobald einer feststeht.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-MVGOOM-00003.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur Pro-Plan-Grundgebühr, keine Nutzungsgebühren in diesem Monat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YL9K6L19-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OpenAI OpCo, LLC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hugo, Wielandstraße 11, 12159 Berlin (runningwithhugo@outlook.de)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. (19%) direkt von OpenAI ausgewiesen (EU OSS VAT EU372041333), kein Reverse Charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-YL9K6L19-0001.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geklärt (19.08.2026): Konto gehört Sandy, 'Hugo' ist ein historischer Nutzername/E-Mail-Alias bei OpenAI, der sich im Nachhinein nicht mehr auf 'Sandra Holm' ändern lässt. Kein falscher Account — nur zur Info für den Steuerberater vermerkt, falls Name/E-Mail auf dem Beleg auffallen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TT0BDQ8S-0003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.06.–21.07.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-TT0BDQ8S-0003.pdf / Receipt-2268-5813.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zusätzliche Position 'Observability Plus' mit $0,00 seit diesem Monat. Zahlungsart nachträglich ergänzt (Update 2026-09-02) anhand Zahlungsbeleg Receipt-2268-5813.pdf.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVGOOM-00005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.05.–22.06.2026 (Nutzung) + 23.06.–22.07.2026 (Pro Plan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-MVGOOM-00005.pdf / Receipt-MVGOOM-00005.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erstmals nennenswerte Nutzungsgebühren (Compute Hours) zusätzlich zur Pro-Plan-Grundgebühr. Zahlungsbeleg (Receipt-MVGOOM-00005.pdf) nachträglich ergänzt (Update 2026-09-02), keine neue Zeile — identischer Betrag/Zeitraum wie diese Rechnung.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TT0BDQ8S-0004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.07.–21.08.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-TT0BDQ8S-0004.pdf / Receipt-2842-3830.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zahlungsart nachträglich ergänzt (Update 2026-09-02) anhand Zahlungsbeleg Receipt-2842-3830.pdf.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVGOOM-00006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.06.–22.07.2026 (Nutzung) + 23.07.–22.08.2026 (Pro Plan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-MVGOOM-00006.pdf / Receipt-MVGOOM-00006.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nutzungsgebühren weiter gestiegen, neu: 'Realtime Peak Connections' $10,00. Rechnung listet 5 verschiedene Projekt-Referenzen, dokumentiert sind nur 2 (Staging + Produktion). Zahlungsbeleg (Receipt-MVGOOM-00006.pdf) nachträglich ergänzt (Update 2026-09-02), keine neue Zeile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVS3312KT5 / Dok. 674170779929</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03.08.–02.09.2026 (Abo-Monat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deine Käufe bei Apple.eml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belege für die Juni- und Juli-Abbuchung dieses Abos fehlen noch (vermutlich auch je ~22 €) — bitte in Apple-Kaufhistorie/Postfach nachsehen und ergänzen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CBBICKXQ-0001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthropic, PBC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandra Holm, Wielandstraße 11, 12159 Berlin, DE STN 89365407818</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. (19%) direkt von Anthropic ausgewiesen (EU VAT IE4276970QH), kein Reverse Charge.</t>
+  </si>
+  <si>
     <t xml:space="preserve">unbekannt (Online-Zahlung)</t>
   </si>
   <si>
-    <t xml:space="preserve">Invoice-TT0BDQ8S-0001.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVGOOM-00003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.05.–22.06.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supabase Pte. Ltd.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Singapur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandra Holm, Wielandstraße 11, Berlin (einfachanfrage@outlook.com)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reverse Charge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reverse Charge — Supabase weist keine USt aus. Sandy startet als Kleinunternehmerin nach §19 UStG (bestätigt 19.08.2026), Gewerbe aber noch nicht angemeldet. Nach Kleinunternehmerregelung i. d. R. keine Vorsteuer ziehbar, aber die USt-Pflicht auf reverse-charge-Leistungen aus dem Ausland (§13b UStG) kann trotzdem bestehen bleiben — das ist keine verbindliche Auskunft von mir, bitte mit Steuerberater final klären, sobald einer feststeht.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-MVGOOM-00003.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nur Pro-Plan-Grundgebühr, keine Nutzungsgebühren in diesem Monat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YL9K6L19-0001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OpenAI OpCo, LLC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hugo, Wielandstraße 11, 12159 Berlin (runningwithhugo@outlook.de)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USt. (19%) direkt von OpenAI ausgewiesen (EU OSS VAT EU372041333), kein Reverse Charge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-YL9K6L19-0001.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geklärt (19.08.2026): Konto gehört Sandy, 'Hugo' ist ein historischer Nutzername/E-Mail-Alias bei OpenAI, der sich im Nachhinein nicht mehr auf 'Sandra Holm' ändern lässt. Kein falscher Account — nur zur Info für den Steuerberater vermerkt, falls Name/E-Mail auf dem Beleg auffallen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TT0BDQ8S-0003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.06.–21.07.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-TT0BDQ8S-0003.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zusätzliche Position 'Observability Plus' mit $0,00 seit diesem Monat.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVGOOM-00005</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.05.–22.06.2026 (Nutzung) + 23.06.–22.07.2026 (Pro Plan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-MVGOOM-00005.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Erstmals nennenswerte Nutzungsgebühren (Compute Hours) zusätzlich zur Pro-Plan-Grundgebühr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TT0BDQ8S-0004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22.07.–21.08.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-TT0BDQ8S-0004.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVGOOM-00006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23.06.–22.07.2026 (Nutzung) + 23.07.–22.08.2026 (Pro Plan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invoice-MVGOOM-00006.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nutzungsgebühren weiter gestiegen, neu: 'Realtime Peak Connections' $10,00. Rechnung listet 5 verschiedene Projekt-Referenzen, dokumentiert sind nur 2 (Staging + Produktion).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVS3312KT5 / Dok. 674170779929</t>
-  </si>
-  <si>
-    <t xml:space="preserve">03.08.–02.09.2026 (Abo-Monat)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deine Käufe bei Apple.eml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belege für die Juni- und Juli-Abbuchung dieses Abos fehlen noch (vermutlich auch je ~22 €) — bitte in Apple-Kaufhistorie/Postfach nachsehen und ergänzen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CBBICKXQ-0001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Anthropic, PBC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandra Holm, Wielandstraße 11, 12159 Berlin, DE STN 89365407818</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USt. (19%) direkt von Anthropic ausgewiesen (EU VAT IE4276970QH), kein Reverse Charge.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Invoice-CBBICKXQ-0001.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Rechnung nennt eine deutsche Steuernummer (DE STN 89365407818) — da laut Sandy noch kein Gewerbe angemeldet ist (Stand 19.08.2026), vermutlich Sandys private Steuer-ID, nicht zwingend eine Geschäfts-Steuernummer. Position heißt 'Prepaid extra usage, Individual plan' — bitte klären: wiederkehrender Posten oder einmaliger Nachkauf von Nutzungsvolumen?</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100185593347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrechnung 26.04.2026 (Vertragszeitraum Domain: 25.04.2026–24.04.2027)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS SE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deutschland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandra Holm, Wielandstr. 11, 12159 Berlin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. (19%) direkt von IONOS ausgewiesen (deutscher Anbieter, USt-IdNr. DE815563912), kein Reverse Charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS Rechnung 2026-04-26 - RG_100185593347.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechnung betrifft ausschließlich die Domain 'einfach-anfrage.com' (Position 1) — das ist NICHT sofortangebot.app, sondern offensichtlich ein anderes/älteres Projekt. Deshalb Sofortangebot-Anteil = 0,00 €. Alle 5 IONOS-Rechnungen (April–August 2026) laufen unter derselben Vertragsnummer 111811442, die mehrere Domains bündelt — bitte im Blick behalten, dass hier nicht versehentlich fremde Projektkosten mitgezählt werden. Neu entdeckt und nachgetragen: Update 2026-09-02.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100187536255</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrechnung 26.05.2026 (Vertragszeiträume: 11.05.2026–10.05.2027 bzw. 22.05.2026–21.05.2027)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS Rechnung 2026-05-26 - RG_100187536255.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechnung betrifft drei fremde Domains ('einfachanfrage.com', 'einfachanfrage-hochzeitsfotografie.de', 'einfachanfrage-tattoo.de') plus deren Registrierungsgebühren — keine davon ist sofortangebot.app. Deshalb Sofortangebot-Anteil = 0,00 €. Neu entdeckt und nachgetragen: Update 2026-09-02.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-013</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100189466040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abrechnung 26.06.2026 (Domain .app + Domain Guard: 08.06.2026–07.06.2027; IONOS Mail Basic 5: 08.06.–07.07.2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. (19%) direkt von IONOS ausgewiesen, kein Reverse Charge. Hinweis für Steuerberater: Die Spalte 'Betrag (EUR)' auf IONOS-Rechnungen zeigt Brutto-Positionsbeträge, obwohl daneben eine MwSt.-Spalte steht — Netto/USt werden nur für die Rechnungssumme insgesamt ausgewiesen, nicht je Zeile. Der Sofortangebot-Anteil (Brutto) wurde deshalb direkt aus den Positionsbeträgen gebildet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS Rechnung 2026-06-26 - RG_100189466040.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erste Rechnung mit sofortangebot.app: Domain .app registriert 08.06.2026 (12,00 € brutto). Sandy hat am 02.09.2026 bestätigt, dass 'Domain Guard' (1,00 € brutto, Privatsphärenschutz) UND 'IONOS Mail Basic 5' (2,50 €/Monat, ab 08.06.2026) ebenfalls zu sofortangebot.app gehören — damit ist die komplette Rechnung (15,50 €) dem Sofortangebot-Anteil zugeordnet. Alle 5 IONOS-Rechnungen laufen unter Vertragsnummer 111811442, die mehrere fremde Domains bündelt (siehe 2026-011/012), die weiterhin ausgeschlossen bleiben. Neu entdeckt: Update 2026-09-02, Zuordnung bestätigt 2026-09-02.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100191208015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08.07.–07.08.2026 (IONOS Mail Basic 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USt. (19%) direkt von IONOS ausgewiesen, kein Reverse Charge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS Rechnung 2026-07-26 - RG_100191208015.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nur Position 'IONOS Mail Basic 5' (2,50 €) — dasselbe Postfach wie in 2026-013. Sandy hat am 02.09.2026 bestätigt, dass es zu sofortangebot.app gehört. Neu entdeckt: Update 2026-09-02, Zuordnung bestätigt 2026-09-02.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TT0BDQ8S-0005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22.08.–21.09.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-TT0BDQ8S-0005.pdf / Receipt-2017-0960.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Weiterhin 'Observability Plus' Position mit $0,00. Zahlungsart über Zahlungsbeleg bestätigt: Visa-Karte endet auf 3991 (gilt rückwirkend auch für 2026-002/005/007, dort ergänzt).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVGOOM-00007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23.07.–22.08.2026 (Nutzung) + 23.08.–22.09.2026 (Pro Plan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invoice-MVGOOM-00007.pdf / Receipt-MVGOOM-00007.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nutzungsgebühren leicht gesunken ggü. Juli ($54,30 → $53,83). Positiv aufgefallen: nur noch 4 Projekt-Referenzen in den Positionen sichtbar (bkldyddstovvkkhpiqiy, ezgyklsigzaowrrpqtpv, qsdbnckgzllyypmkmzhc, yqlledouhfovytifeekd) — die fünfte aus den Vormonaten ('ytvysmwepajatcdhkgup') taucht hier nicht mehr auf. Könnte bedeuten, dass ein ungenutztes Projekt zwischenzeitlich entfernt wurde (siehe offener Punkt '5 vs. 2 dokumentierte Projekte').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100192688572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08.08.–07.09.2026 (IONOS Mail Basic 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IONOS Rechnung 2026-08-26 - RG_100192688572.pdf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wie Juli: nur 'IONOS Mail Basic 5' (2,50 €). Sandy hat am 02.09.2026 bestätigt, dass es zu sofortangebot.app gehört (siehe 2026-013/014).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Monatsverlauf laufende Kosten</t>
   </si>
   <si>
@@ -723,7 +909,7 @@
     <t xml:space="preserve">1) Kostenübersicht — ein Dienst pro Zeile: aktuellster Betrag, Rhythmus, USt-Behandlung, Status.</t>
   </si>
   <si>
-    <t xml:space="preserve">2) Rechnungsjournal — die eigentliche Beleg-Ebene: eine Zeile pro Rechnung, mit allem, was für die Buchhaltung zählt (Rechnungsnummer, Leistungszeitraum, Netto/USt/Brutto, Reverse-Charge-Kennzeichnung, Zahlungsart, Verweis auf die Beleg-Datei im Ordner). Neue Belege bitte als neue Zeile anhängen, nie bestehende Zeilen überschreiben (Nachvollziehbarkeit/GoBD-Grundsatz).</t>
+    <t xml:space="preserve">2) Rechnungsjournal — die eigentliche Beleg-Ebene: eine Zeile pro Rechnung, mit allem, was für die Buchhaltung zählt (Rechnungsnummer, Leistungszeitraum, Netto/USt/Brutto, Reverse-Charge-Kennzeichnung, Zahlungsart, Verweis auf die Beleg-Datei im Ordner). Neue Belege bitte als neue Zeile anhängen, nie bestehende Zeilen überschreiben (Nachvollziehbarkeit/GoBD-Grundsatz). Seit 2026-09-02 zusätzlich Spalte 'Sofortangebot-Anteil (Brutto)': bei Rechnungen, die mehrere Domains/Projekte bündeln (aktuell nur die IONOS-Domainrechnungen), steht in 'Brutto-Betrag' weiterhin die volle Original-Rechnungssumme (GoBD-Vollständigkeit), aber in 'Sofortangebot-Anteil' nur der Teil, der tatsächlich zu Sofortangebot gehört. Monatsverlauf rechnet mit dem Anteil, nicht mit dem vollen Brutto-Betrag.</t>
   </si>
   <si>
     <t xml:space="preserve">3) Monatsverlauf — zieht die Beträge per Formel automatisch aus dem Rechnungsjournal (nach Monat, Dienst, Währung). Aktualisiert sich von selbst, sobald neue Journal-Zeilen dazukommen.</t>
@@ -738,28 +924,31 @@
     <t xml:space="preserve">Sandy hat noch KEIN Gewerbe angemeldet, startet aber als Kleinunternehmerin nach §19 UStG (bestätigt). Alle bisherigen Belege stammen damit aus der Zeit vor der offiziellen Gründung — das ist normal und die Kosten lassen sich in der Regel nachträglich als 'vorweggenommene Betriebsausgaben' geltend machen, sobald das Gewerbe angemeldet ist. Wichtig dafür ist genau das, was dieses Journal leistet: ein lückenloser, nachvollziehbarer Beleg-Nachweis. Eine Detailfrage bleibt offen, die ich bewusst nicht selbst beantworte: Wie sind die Reverse-Charge-Rechnungen (Supabase) für eine Kleinunternehmerin zu behandeln — meines Wissens kann die USt-Pflicht auf im Ausland eingekaufte Leistungen (§13b UStG) auch für Kleinunternehmer bestehen bleiben, während der Vorsteuerabzug bei den anderen Diensten (Vercel, OpenAI, Anthropic, Apple) i. d. R. entfällt, weil keine Regelbesteuerung vorliegt — das ist aber keine verbindliche Auskunft von mir. Bitte mit dem Steuerberater klären, sobald einer feststeht — bis dahin im Journal bewusst vorläufig dokumentiert.</t>
   </si>
   <si>
-    <t xml:space="preserve">Auffälligkeiten aus den bisherigen 10 Belegen (Stand 2026-08-19) — bitte von Sandy klären</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Supabase: Kosten steigen (Mai $25,00 → Juni $49,97 → Juli $54,30). Belege zeigen 5 verschiedene Projekt-Referenzen, dokumentiert sind nur 2 (Staging + Produktion). Werden alle 5 gebraucht?</t>
+    <t xml:space="preserve">Auffälligkeiten aus den bisherigen 17 Belegen (Stand 2026-09-02) — bitte von Sandy klären</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Supabase: Kosten seit Mai gestiegen ($25,00 → $49,97 → $54,30), im August leicht gesunken auf $53,83. Weiterhin 5 verschiedene Projekt-Referenzen in älteren Belegen, dokumentiert sind nur 2 (Staging + Produktion) — im August-Beleg (MVGOOM-00007) taucht eine der 5 Referenzen ('ytvysmwepajatcdhkgup') erstmals nicht mehr auf. Werden die verbleibenden 4 alle gebraucht?</t>
   </si>
   <si>
     <t xml:space="preserve">• Zwei offenbar getrennte Claude-Positionen: direkte Anthropic-Rechnung (Geschäftsadresse) UND Claude-Pro-Abo über Apple/iTunes (22 €/Monat, andere Adresse, PayPal). Geschäftlich oder privat?</t>
   </si>
   <si>
-    <t xml:space="preserve">• Claude-Pro-Apple-Abo: Belege für Juni und Juli fehlen (nur Mai und August vorhanden) — bitte in der Apple-Kaufhistorie nachsehen und ergänzen, damit der Monatsverlauf vollständig ist.</t>
+    <t xml:space="preserve">• Claude-Pro-Apple-Abo: Belege für Juni und Juli fehlen weiterhin (nur Mai und August vorhanden) — bitte in der Apple-Kaufhistorie nachsehen und ergänzen, damit der Monatsverlauf vollständig ist.</t>
   </si>
   <si>
     <t xml:space="preserve">• Zwei unterschiedliche Adressen für Sandra Holm (Wielandstraße 11 vs. Krampasplatz 4b) — vermutlich alt/neu, bitte kurz bestätigen.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Genaues Datum der geplanten Gewerbeanmeldung? Hilft bei der sauberen Abgrenzung, welche Belege als vorweggenommene Betriebsausgaben zählen.</t>
+    <t xml:space="preserve">• Genaues Datum der geplanten Gewerbeanmeldung? Hilft bei der sauberen Abgrenzung, welche Belege als vorweggenommene Betriebsausgaben zählen. Zusätzlich jetzt relevant: Sandy erwägt statt/neben dem Kleingewerbe eine UG (haftungsbeschränkt) — betrifft auch die Buchführungspflichten, siehe Update im Koordinations-Dokument.</t>
   </si>
   <si>
     <t xml:space="preserve">• Wie sind die Supabase-Reverse-Charge-Rechnungen für eine Kleinunternehmerin (§19 UStG) zu behandeln (siehe Absatz oben)? — mit Steuerberater klären, sobald einer feststeht.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Noch keine Belege gefunden für: Resend, Domain sofortangebot.app, Sentry, GitHub-Plan.</t>
+    <t xml:space="preserve">• IONOS-Domainrechnungen (Vertragsnummer 111811442) bündeln mehrere Domains — nur sofortangebot.app zählt für Sofortangebot (siehe Journal 2026-011 bis 2026-017 und Spalte 'Sofortangebot-Anteil'). Geklärt (Sandy, 02.09.2026): 'Domain Guard' (1,00 €, Privatsphärenschutz) und 'IONOS Mail Basic 5' (2,50 €/Monat) gehören beide zu sofortangebot.app — entsprechend im Anteil berücksichtigt. Die übrigen, klar fremden Domains auf denselben Rechnungen bleiben weiterhin ausgeschlossen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Noch keine Belege gefunden für: Resend, Sentry, GitHub-Plan.</t>
   </si>
   <si>
     <t xml:space="preserve">• Anthropic-Direktrechnung: einmaliger Nachkauf oder wiederkehrender Posten?</t>
@@ -1028,6 +1217,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1049,10 +1242,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1477,7 +1666,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -1488,7 +1677,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>54.3</v>
+        <v>53.83</v>
       </c>
       <c r="E5" s="4" t="s">
         <v>14</v>
@@ -1649,7 +1838,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="115.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>50</v>
       </c>
@@ -1657,9 +1846,11 @@
         <v>51</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="9"/>
+        <v>35</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>2.5</v>
+      </c>
       <c r="E11" s="4" t="s">
         <v>52</v>
       </c>
@@ -1667,21 +1858,21 @@
         <v>53</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>48</v>
+        <v>54</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>47</v>
@@ -1700,22 +1891,22 @@
         <v>48</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>47</v>
       </c>
       <c r="D13" s="9"/>
       <c r="E13" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>29</v>
@@ -1724,44 +1915,44 @@
         <v>29</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>47</v>
       </c>
       <c r="D14" s="9"/>
       <c r="E14" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>29</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="11"/>
+      <c r="D15" s="12"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
@@ -1772,7 +1963,7 @@
       <c r="A16" s="10"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
-      <c r="D16" s="11"/>
+      <c r="D16" s="12"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
@@ -1780,40 +1971,40 @@
       <c r="I16" s="4"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14" t="n">
+      <c r="A18" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="15" t="n">
         <f aca="false">SUMIF(C5:C16,"USD",D5:D16)</f>
-        <v>149.5</v>
-      </c>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
+        <v>149.03</v>
+      </c>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+      <c r="I18" s="14"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="15" t="n">
+      <c r="A19" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="16" t="n">
         <f aca="false">SUMIF(C5:C16,"EUR",D5:D16)</f>
-        <v>22</v>
-      </c>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
+        <v>24.5</v>
+      </c>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+      <c r="I19" s="14"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -1860,15 +2051,16 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1891,7 +2083,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1914,141 +2106,147 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>2</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B5" s="16" t="n">
+        <v>92</v>
+      </c>
+      <c r="B5" s="17" t="n">
         <v>46146</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>33</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I5" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J5" s="17" t="n">
+      <c r="J5" s="11" t="n">
         <v>18.49</v>
       </c>
       <c r="K5" s="18" t="n">
         <v>0.19</v>
       </c>
-      <c r="L5" s="17" t="n">
+      <c r="L5" s="11" t="n">
         <v>3.51</v>
       </c>
-      <c r="M5" s="17" t="n">
+      <c r="M5" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="N5" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="O5" s="19" t="n">
+      <c r="N5" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="P5" s="19" t="n">
         <f aca="false">M5</f>
         <v>22</v>
       </c>
-      <c r="P5" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="Q5" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="R5" s="20" t="s">
         <v>99</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="S5" s="20" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="B6" s="16" t="n">
+        <v>102</v>
+      </c>
+      <c r="B6" s="17" t="n">
         <v>46164</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>13</v>
@@ -2065,42 +2263,47 @@
       <c r="M6" s="7" t="n">
         <v>23.8</v>
       </c>
-      <c r="N6" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O6" s="21"/>
-      <c r="P6" s="4" t="s">
-        <v>107</v>
-      </c>
+      <c r="N6" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P6" s="21"/>
       <c r="Q6" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="R6" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="S6" s="20" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B7" s="16" t="n">
+        <v>112</v>
+      </c>
+      <c r="B7" s="17" t="n">
         <v>46165</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I7" s="4" t="s">
         <v>13</v>
@@ -2109,7 +2312,7 @@
         <v>25</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="L7" s="7" t="n">
         <v>0</v>
@@ -2117,44 +2320,47 @@
       <c r="M7" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="N7" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="O7" s="21"/>
-      <c r="P7" s="4" t="s">
+      <c r="N7" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Q7" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="R7" s="20" t="s">
-        <v>118</v>
+      <c r="R7" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="S7" s="20" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="B8" s="16" t="n">
+        <v>122</v>
+      </c>
+      <c r="B8" s="17" t="n">
         <v>46187</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>41</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I8" s="4" t="s">
         <v>13</v>
@@ -2171,44 +2377,47 @@
       <c r="M8" s="7" t="n">
         <v>17.85</v>
       </c>
-      <c r="N8" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="O8" s="21"/>
-      <c r="P8" s="4" t="s">
+      <c r="N8" s="7" t="n">
+        <v>17.85</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Q8" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="R8" s="20" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="R8" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="S8" s="20" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="B9" s="16" t="n">
+        <v>130</v>
+      </c>
+      <c r="B9" s="17" t="n">
         <v>46195</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>13</v>
@@ -2225,44 +2434,47 @@
       <c r="M9" s="7" t="n">
         <v>23.8</v>
       </c>
-      <c r="N9" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O9" s="21"/>
-      <c r="P9" s="4" t="s">
-        <v>107</v>
-      </c>
+      <c r="N9" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P9" s="21"/>
       <c r="Q9" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="R9" s="20" t="s">
-        <v>131</v>
+        <v>109</v>
+      </c>
+      <c r="R9" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="S9" s="20" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B10" s="16" t="n">
+        <v>135</v>
+      </c>
+      <c r="B10" s="17" t="n">
         <v>46196</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>13</v>
@@ -2271,7 +2483,7 @@
         <v>49.97</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="L10" s="7" t="n">
         <v>0</v>
@@ -2279,44 +2491,47 @@
       <c r="M10" s="7" t="n">
         <v>49.97</v>
       </c>
-      <c r="N10" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="O10" s="21"/>
-      <c r="P10" s="4" t="s">
+      <c r="N10" s="7" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Q10" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="R10" s="20" t="s">
-        <v>136</v>
+      <c r="R10" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="S10" s="20" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="B11" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="B11" s="17" t="n">
         <v>46225</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>13</v>
@@ -2333,42 +2548,47 @@
       <c r="M11" s="7" t="n">
         <v>23.8</v>
       </c>
-      <c r="N11" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="O11" s="21"/>
-      <c r="P11" s="4" t="s">
-        <v>107</v>
-      </c>
+      <c r="N11" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P11" s="21"/>
       <c r="Q11" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="R11" s="4"/>
+        <v>109</v>
+      </c>
+      <c r="R11" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="S11" s="20" t="s">
+        <v>144</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="B12" s="16" t="n">
+        <v>145</v>
+      </c>
+      <c r="B12" s="17" t="n">
         <v>46226</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="G12" s="4" t="s">
         <v>11</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>13</v>
@@ -2377,7 +2597,7 @@
         <v>54.3</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="L12" s="7" t="n">
         <v>0</v>
@@ -2385,101 +2605,107 @@
       <c r="M12" s="7" t="n">
         <v>54.3</v>
       </c>
-      <c r="N12" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="O12" s="21"/>
-      <c r="P12" s="4" t="s">
+      <c r="N12" s="7" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P12" s="21"/>
+      <c r="Q12" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="Q12" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="R12" s="20" t="s">
-        <v>145</v>
+      <c r="R12" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="S12" s="20" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="B13" s="16" t="n">
+        <v>150</v>
+      </c>
+      <c r="B13" s="17" t="n">
         <v>46237</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G13" s="4" t="s">
         <v>33</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="J13" s="17" t="n">
+      <c r="J13" s="11" t="n">
         <v>18.49</v>
       </c>
       <c r="K13" s="18" t="n">
         <v>0.19</v>
       </c>
-      <c r="L13" s="17" t="n">
+      <c r="L13" s="11" t="n">
         <v>3.51</v>
       </c>
-      <c r="M13" s="17" t="n">
+      <c r="M13" s="11" t="n">
         <v>22</v>
       </c>
-      <c r="N13" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="O13" s="19" t="n">
+      <c r="N13" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="P13" s="19" t="n">
         <f aca="false">M13</f>
         <v>22</v>
       </c>
-      <c r="P13" s="4" t="s">
-        <v>97</v>
-      </c>
       <c r="Q13" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="R13" s="20" t="s">
-        <v>150</v>
+        <v>99</v>
+      </c>
+      <c r="R13" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="S13" s="20" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="B14" s="16" t="n">
+        <v>155</v>
+      </c>
+      <c r="B14" s="17" t="n">
         <v>46251</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G14" s="4" t="s">
         <v>26</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>13</v>
@@ -2496,159 +2722,436 @@
       <c r="M14" s="7" t="n">
         <v>53.55</v>
       </c>
-      <c r="N14" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="O14" s="21"/>
-      <c r="P14" s="4" t="s">
+      <c r="N14" s="7" t="n">
+        <v>53.55</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="R14" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="S14" s="20" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>46138</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L15" s="11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M15" s="11" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P15" s="19" t="n">
+        <f aca="false">M15</f>
+        <v>0.96</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="R15" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="S15" s="20" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>46168</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>27.73</v>
+      </c>
+      <c r="K16" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L16" s="11" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="M16" s="11" t="n">
+        <v>33</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="P16" s="19" t="n">
+        <f aca="false">M16</f>
+        <v>33</v>
+      </c>
+      <c r="Q16" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="S16" s="20" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="191.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B17" s="17" t="n">
+        <v>46199</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>13.03</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L17" s="11" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="M17" s="11" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="N17" s="11" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="P17" s="19" t="n">
+        <f aca="false">M17</f>
+        <v>15.5</v>
+      </c>
+      <c r="Q17" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="S17" s="20" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>46229</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="K18" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L18" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M18" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N18" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="P18" s="19" t="n">
+        <f aca="false">M18</f>
+        <v>2.5</v>
+      </c>
+      <c r="Q18" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="S18" s="20" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>46256</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="Q14" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="R14" s="20" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="22"/>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="22"/>
-      <c r="R15" s="22"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="22"/>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
-      <c r="R16" s="22"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="22"/>
-      <c r="R17" s="22"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="22"/>
-      <c r="P18" s="22"/>
-      <c r="Q18" s="22"/>
-      <c r="R18" s="22"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
-      <c r="P19" s="22"/>
-      <c r="Q19" s="22"/>
-      <c r="R19" s="22"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="22"/>
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="22"/>
-      <c r="P20" s="22"/>
-      <c r="Q20" s="22"/>
-      <c r="R20" s="22"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22"/>
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="22"/>
-      <c r="P21" s="22"/>
-      <c r="Q21" s="22"/>
-      <c r="R21" s="22"/>
+      <c r="I19" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="K19" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L19" s="7" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M19" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="N19" s="7" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="R19" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="S19" s="20" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="179.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" s="17" t="n">
+        <v>46257</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="L20" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="7" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="N20" s="7" t="n">
+        <v>53.83</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="R20" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="S20" s="20" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B21" s="17" t="n">
+        <v>46260</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J21" s="11" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="K21" s="18" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="L21" s="11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="M21" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N21" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="P21" s="19" t="n">
+        <f aca="false">M21</f>
+        <v>2.5</v>
+      </c>
+      <c r="Q21" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="R21" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="S21" s="20" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22"/>
@@ -2669,6 +3172,7 @@
       <c r="P22" s="22"/>
       <c r="Q22" s="22"/>
       <c r="R22" s="22"/>
+      <c r="S22" s="22"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22"/>
@@ -2689,6 +3193,7 @@
       <c r="P23" s="22"/>
       <c r="Q23" s="22"/>
       <c r="R23" s="22"/>
+      <c r="S23" s="22"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="22"/>
@@ -2709,6 +3214,7 @@
       <c r="P24" s="22"/>
       <c r="Q24" s="22"/>
       <c r="R24" s="22"/>
+      <c r="S24" s="22"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22"/>
@@ -2729,6 +3235,7 @@
       <c r="P25" s="22"/>
       <c r="Q25" s="22"/>
       <c r="R25" s="22"/>
+      <c r="S25" s="22"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="22"/>
@@ -2749,6 +3256,7 @@
       <c r="P26" s="22"/>
       <c r="Q26" s="22"/>
       <c r="R26" s="22"/>
+      <c r="S26" s="22"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22"/>
@@ -2769,6 +3277,7 @@
       <c r="P27" s="22"/>
       <c r="Q27" s="22"/>
       <c r="R27" s="22"/>
+      <c r="S27" s="22"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="22"/>
@@ -2789,6 +3298,7 @@
       <c r="P28" s="22"/>
       <c r="Q28" s="22"/>
       <c r="R28" s="22"/>
+      <c r="S28" s="22"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="22"/>
@@ -2809,6 +3319,7 @@
       <c r="P29" s="22"/>
       <c r="Q29" s="22"/>
       <c r="R29" s="22"/>
+      <c r="S29" s="22"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22"/>
@@ -2829,6 +3340,7 @@
       <c r="P30" s="22"/>
       <c r="Q30" s="22"/>
       <c r="R30" s="22"/>
+      <c r="S30" s="22"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="22"/>
@@ -2849,6 +3361,7 @@
       <c r="P31" s="22"/>
       <c r="Q31" s="22"/>
       <c r="R31" s="22"/>
+      <c r="S31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="22"/>
@@ -2869,6 +3382,7 @@
       <c r="P32" s="22"/>
       <c r="Q32" s="22"/>
       <c r="R32" s="22"/>
+      <c r="S32" s="22"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22"/>
@@ -2889,6 +3403,7 @@
       <c r="P33" s="22"/>
       <c r="Q33" s="22"/>
       <c r="R33" s="22"/>
+      <c r="S33" s="22"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="22"/>
@@ -2909,6 +3424,7 @@
       <c r="P34" s="22"/>
       <c r="Q34" s="22"/>
       <c r="R34" s="22"/>
+      <c r="S34" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2941,7 +3457,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>204</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2955,7 +3471,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>159</v>
+        <v>205</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2972,31 +3488,31 @@
         <v>2</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>160</v>
+        <v>206</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>161</v>
+        <v>207</v>
       </c>
       <c r="D4" s="24" t="s">
-        <v>162</v>
+        <v>208</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>163</v>
+        <v>209</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>164</v>
+        <v>210</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>165</v>
+        <v>211</v>
       </c>
       <c r="H4" s="24" t="s">
-        <v>166</v>
+        <v>212</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>167</v>
+        <v>213</v>
       </c>
       <c r="J4" s="25" t="s">
-        <v>168</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3004,40 +3520,40 @@
         <v>11</v>
       </c>
       <c r="B5" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
         <v>25</v>
       </c>
       <c r="C5" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
         <v>49.97</v>
       </c>
       <c r="D5" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
         <v>54.3</v>
       </c>
-      <c r="E5" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+      <c r="E5" s="27" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <v>53.83</v>
+      </c>
+      <c r="F5" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
         <v/>
       </c>
-      <c r="F5" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+      <c r="G5" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
         <v/>
       </c>
-      <c r="G5" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+      <c r="H5" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
         <v/>
       </c>
-      <c r="H5" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
-        <v/>
-      </c>
       <c r="I5" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A5,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
         <v/>
       </c>
       <c r="J5" s="28" t="n">
         <f aca="false">SUM(B5:I5)</f>
-        <v>129.27</v>
+        <v>183.1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3045,40 +3561,40 @@
         <v>19</v>
       </c>
       <c r="B6" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
         <v>23.8</v>
       </c>
       <c r="C6" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
         <v>23.8</v>
       </c>
       <c r="D6" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
         <v>23.8</v>
       </c>
-      <c r="E6" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+      <c r="E6" s="27" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <v>23.8</v>
+      </c>
+      <c r="F6" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
         <v/>
       </c>
-      <c r="F6" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+      <c r="G6" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
         <v/>
       </c>
-      <c r="G6" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+      <c r="H6" s="27" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
         <v/>
       </c>
-      <c r="H6" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
-        <v/>
-      </c>
       <c r="I6" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A6,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
         <v/>
       </c>
       <c r="J6" s="28" t="n">
         <f aca="false">SUM(B6:I6)</f>
-        <v>71.4</v>
+        <v>95.2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3086,35 +3602,35 @@
         <v>26</v>
       </c>
       <c r="B7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
         <v/>
       </c>
       <c r="C7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
         <v/>
       </c>
       <c r="D7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
         <v/>
       </c>
       <c r="E7" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
         <v>53.55</v>
       </c>
       <c r="F7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
         <v/>
       </c>
       <c r="G7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
         <v/>
       </c>
       <c r="H7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
         <v/>
       </c>
       <c r="I7" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A7,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
         <v/>
       </c>
       <c r="J7" s="28" t="n">
@@ -3127,35 +3643,35 @@
         <v>33</v>
       </c>
       <c r="B8" s="29" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
         <v>22</v>
       </c>
       <c r="C8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
         <v/>
       </c>
       <c r="D8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
         <v/>
       </c>
       <c r="E8" s="29" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
         <v>22</v>
       </c>
       <c r="F8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
         <v/>
       </c>
       <c r="G8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
         <v/>
       </c>
       <c r="H8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
         <v/>
       </c>
       <c r="I8" s="29" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A8,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
         <v/>
       </c>
       <c r="J8" s="30" t="n">
@@ -3168,35 +3684,35 @@
         <v>41</v>
       </c>
       <c r="B9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
         <v/>
       </c>
       <c r="C9" s="27" t="n">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
         <v>17.85</v>
       </c>
       <c r="D9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
         <v/>
       </c>
       <c r="E9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
         <v/>
       </c>
       <c r="F9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
         <v/>
       </c>
       <c r="G9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
         <v/>
       </c>
       <c r="H9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
         <v/>
       </c>
       <c r="I9" s="27" t="str">
-        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$M$5:$M$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A9,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
         <v/>
       </c>
       <c r="J9" s="28" t="n">
@@ -3225,22 +3741,46 @@
       <c r="A11" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="32" t="n">
+      <c r="B11" s="29" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,5,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,6,1)))</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,6,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,7,1)))</f>
+        <v>15.5</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,7,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,8,1)))</f>
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="29" t="n">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,8,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,9,1)))</f>
+        <v>2.5</v>
+      </c>
+      <c r="F11" s="29" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,9,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,10,1)))</f>
+        <v/>
+      </c>
+      <c r="G11" s="29" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,10,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,11,1)))</f>
+        <v/>
+      </c>
+      <c r="H11" s="29" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,11,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2026,12,1)))</f>
+        <v/>
+      </c>
+      <c r="I11" s="29" t="str">
+        <f aca="false">IF(COUNTIFS(Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1))=0,"",SUMIFS(Rechnungsjournal!$N$5:$N$34,Rechnungsjournal!$G$5:$G$34,$A11,Rechnungsjournal!$B$5:$B$34,"&gt;="&amp;DATE(2026,12,1),Rechnungsjournal!$B$5:$B$34,"&lt;"&amp;DATE(2027,1,1)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="30" t="n">
         <f aca="false">SUM(B11:I11)</f>
-        <v>0</v>
+        <v>20.5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="26" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" s="31"/>
       <c r="C12" s="31"/>
@@ -3257,7 +3797,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="31"/>
       <c r="C13" s="31"/>
@@ -3274,7 +3814,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="26" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B14" s="31"/>
       <c r="C14" s="31"/>
@@ -3290,77 +3830,77 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="B16" s="14" t="n">
+      <c r="A16" s="13" t="s">
+        <v>215</v>
+      </c>
+      <c r="B16" s="15" t="n">
         <f aca="false">IF(B5="",0,B5)+IF(B6="",0,B6)+IF(B7="",0,B7)+IF(B9="",0,B9)</f>
         <v>48.8</v>
       </c>
-      <c r="C16" s="14" t="n">
+      <c r="C16" s="15" t="n">
         <f aca="false">IF(C5="",0,C5)+IF(C6="",0,C6)+IF(C7="",0,C7)+IF(C9="",0,C9)</f>
         <v>91.62</v>
       </c>
-      <c r="D16" s="14" t="n">
+      <c r="D16" s="15" t="n">
         <f aca="false">IF(D5="",0,D5)+IF(D6="",0,D6)+IF(D7="",0,D7)+IF(D9="",0,D9)</f>
         <v>78.1</v>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <f aca="false">IF(E5="",0,E5)+IF(E6="",0,E6)+IF(E7="",0,E7)+IF(E9="",0,E9)</f>
-        <v>53.55</v>
-      </c>
-      <c r="F16" s="14" t="n">
+        <v>131.18</v>
+      </c>
+      <c r="F16" s="15" t="n">
         <f aca="false">IF(F5="",0,F5)+IF(F6="",0,F6)+IF(F7="",0,F7)+IF(F9="",0,F9)</f>
         <v>0</v>
       </c>
-      <c r="G16" s="14" t="n">
+      <c r="G16" s="15" t="n">
         <f aca="false">IF(G5="",0,G5)+IF(G6="",0,G6)+IF(G7="",0,G7)+IF(G9="",0,G9)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="14" t="n">
+      <c r="H16" s="15" t="n">
         <f aca="false">IF(H5="",0,H5)+IF(H6="",0,H6)+IF(H7="",0,H7)+IF(H9="",0,H9)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="14" t="n">
+      <c r="I16" s="15" t="n">
         <f aca="false">IF(I5="",0,I5)+IF(I6="",0,I6)+IF(I7="",0,I7)+IF(I9="",0,I9)</f>
         <v>0</v>
       </c>
       <c r="J16" s="33"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="B17" s="15" t="n">
-        <f aca="false">IF(B8="",0,B8)</f>
+      <c r="A17" s="13" t="s">
+        <v>216</v>
+      </c>
+      <c r="B17" s="16" t="n">
+        <f aca="false">IF(B8="",0,B8)+IF(B11="",0,B11)</f>
         <v>22</v>
       </c>
-      <c r="C17" s="15" t="n">
-        <f aca="false">IF(C8="",0,C8)</f>
+      <c r="C17" s="16" t="n">
+        <f aca="false">IF(C8="",0,C8)+IF(C11="",0,C11)</f>
+        <v>15.5</v>
+      </c>
+      <c r="D17" s="16" t="n">
+        <f aca="false">IF(D8="",0,D8)+IF(D11="",0,D11)</f>
+        <v>2.5</v>
+      </c>
+      <c r="E17" s="16" t="n">
+        <f aca="false">IF(E8="",0,E8)+IF(E11="",0,E11)</f>
+        <v>24.5</v>
+      </c>
+      <c r="F17" s="16" t="n">
+        <f aca="false">IF(F8="",0,F8)+IF(F11="",0,F11)</f>
         <v>0</v>
       </c>
-      <c r="D17" s="15" t="n">
-        <f aca="false">IF(D8="",0,D8)</f>
+      <c r="G17" s="16" t="n">
+        <f aca="false">IF(G8="",0,G8)+IF(G11="",0,G11)</f>
         <v>0</v>
       </c>
-      <c r="E17" s="15" t="n">
-        <f aca="false">IF(E8="",0,E8)</f>
-        <v>22</v>
-      </c>
-      <c r="F17" s="15" t="n">
-        <f aca="false">IF(F8="",0,F8)</f>
+      <c r="H17" s="16" t="n">
+        <f aca="false">IF(H8="",0,H8)+IF(H11="",0,H11)</f>
         <v>0</v>
       </c>
-      <c r="G17" s="15" t="n">
-        <f aca="false">IF(G8="",0,G8)</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="15" t="n">
-        <f aca="false">IF(H8="",0,H8)</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="15" t="n">
-        <f aca="false">IF(I8="",0,I8)</f>
+      <c r="I17" s="16" t="n">
+        <f aca="false">IF(I8="",0,I8)+IF(I11="",0,I11)</f>
         <v>0</v>
       </c>
       <c r="J17" s="33"/>
@@ -3385,7 +3925,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
@@ -3393,137 +3933,142 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="34" t="s">
-        <v>171</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>172</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>173</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="s">
-        <v>174</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="37" t="s">
-        <v>175</v>
+        <v>221</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="38" t="s">
-        <v>176</v>
+        <v>222</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
-        <v>177</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="40" t="s">
-        <v>178</v>
+        <v>224</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="41" t="s">
-        <v>179</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="35" t="s">
-        <v>180</v>
+        <v>226</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>182</v>
+        <v>228</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="s">
-        <v>183</v>
+        <v>229</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="36" t="s">
-        <v>184</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="35" t="s">
-        <v>185</v>
+        <v>231</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="141" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="36" t="s">
-        <v>186</v>
+        <v>232</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="35" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="36" t="s">
-        <v>188</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="36" t="s">
-        <v>189</v>
+        <v>235</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="36" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="36" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="36" t="s">
-        <v>192</v>
+        <v>238</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="36" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="36" t="s">
-        <v>194</v>
+        <v>240</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="36" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="36" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="42" t="s">
-        <v>197</v>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="36" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="42" t="s">
+        <v>244</v>
       </c>
     </row>
   </sheetData>

</xml_diff>